<commit_message>
Fix rerun outputs and model-averaging summaries
This patch corrects the rerun workflow and refreshed outputs after the model re-fit: it preserves natural b_spatial column order, updates Delta_wAIC<2 selection tables, adds WAIC rescoring summaries, and refreshes convergence/master summaries to match the current rerun code. It also fixes the cluster-density calculation to use model-average group size instead of the observed mean, rebuilds abundance maps with extrapolation summaries and proper grid-level abundance pooling, and removes stale inclusion-probability plots and old full-candidate tables.
</commit_message>
<xml_diff>
--- a/Results/model_summary/Model_Convergence_and_Parameters_Summary.xlsx
+++ b/Results/model_summary/Model_Convergence_and_Parameters_Summary.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="J18">
-        <v>1.0005</v>
+        <v>1.002</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Fully Converged (Rhat &lt; 1.05)</t>
+          <t>Fully Converged (Rhat &lt; 1.05; CAR nodes &lt; 1.10)</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="G51">
-        <v>8.493381812959483E-19</v>
+        <v>-1.517397255574344E-18</v>
       </c>
       <c r="H51">
         <v>0.8188573043708586</v>
@@ -7712,7 +7712,7 @@
         </is>
       </c>
       <c r="G101">
-        <v>-1.285524446116878E-18</v>
+        <v>1.559624645199692E-18</v>
       </c>
       <c r="H101">
         <v>0.8248587692439722</v>
@@ -10812,7 +10812,7 @@
         </is>
       </c>
       <c r="G151">
-        <v>-1.438137686700435E-18</v>
+        <v>1.763168939546332E-18</v>
       </c>
       <c r="H151">
         <v>0.8168501149958796</v>
@@ -13912,7 +13912,7 @@
         </is>
       </c>
       <c r="G201">
-        <v>1.29370184219047E-18</v>
+        <v>-7.262319364454845E-19</v>
       </c>
       <c r="H201">
         <v>0.8239738484413143</v>
@@ -16236,7 +16236,7 @@
         </is>
       </c>
       <c r="G37">
-        <v>-1.49369270259974E-18</v>
+        <v>-1.387692418842715E-18</v>
       </c>
       <c r="H37">
         <v>0.7433540727429683</v>
@@ -18468,7 +18468,7 @@
         </is>
       </c>
       <c r="G73">
-        <v>-2.242018901703907E-18</v>
+        <v>-2.090354742842862E-18</v>
       </c>
       <c r="H73">
         <v>0.732442390580071</v>
@@ -20700,7 +20700,7 @@
         </is>
       </c>
       <c r="G109">
-        <v>-2.844906198363889E-19</v>
+        <v>-2.058652714500355E-19</v>
       </c>
       <c r="H109">
         <v>0.7331751620456304</v>
@@ -23892,7 +23892,7 @@
         </is>
       </c>
       <c r="G51">
-        <v>-2.688907637252341E-18</v>
+        <v>-1.806169988206146E-18</v>
       </c>
       <c r="H51">
         <v>0.7579521381039943</v>
@@ -26992,7 +26992,7 @@
         </is>
       </c>
       <c r="G101">
-        <v>3.328506067151669E-18</v>
+        <v>3.468421403931183E-18</v>
       </c>
       <c r="H101">
         <v>0.7408906870256157</v>
@@ -38926,7 +38926,7 @@
         </is>
       </c>
       <c r="G192">
-        <v>1.890246933974894E-19</v>
+        <v>1.434687707168837E-19</v>
       </c>
       <c r="H192">
         <v>0.3427436471156993</v>
@@ -42118,7 +42118,7 @@
         </is>
       </c>
       <c r="G51">
-        <v>-4.478316324966885E-19</v>
+        <v>-2.303974596708119E-19</v>
       </c>
       <c r="H51">
         <v>0.6600370165826395</v>
@@ -45218,7 +45218,7 @@
         </is>
       </c>
       <c r="G101">
-        <v>-2.114482109475837E-18</v>
+        <v>-2.159603973453967E-18</v>
       </c>
       <c r="H101">
         <v>0.6564527138742384</v>

</xml_diff>